<commit_message>
revisions to the manuscript
</commit_message>
<xml_diff>
--- a/Data/manuscript_output_moe/uninsured_CCdistrict.xlsx
+++ b/Data/manuscript_output_moe/uninsured_CCdistrict.xlsx
@@ -1,89 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drexel0-my.sharepoint.com/personal/tr842_drexel_edu/Documents/Github_repositories/ACTIVE_Council District Project Repository 05.2026/philadelphia-council-districts-and-health/Data/manuscript_output_moe/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4E66FDCE8F79A8D366075C52F38B5A32EC8F98BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3507E22-75A3-CC40-AE26-BA43B9B2B892}"/>
   <bookViews>
-    <workbookView xWindow="-6700" yWindow="2620" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>DISTRICT</t>
-  </si>
-  <si>
-    <t>CD_uninsurance</t>
-  </si>
-  <si>
-    <t>CD_uninsurance_moe</t>
-  </si>
-  <si>
-    <t>CD_pop</t>
-  </si>
-  <si>
-    <t>percentage_uninsured</t>
-  </si>
-  <si>
-    <t>percentage_uninsured_moe</t>
-  </si>
-  <si>
-    <t>within_sd</t>
-  </si>
-  <si>
-    <t>between_sd</t>
-  </si>
-  <si>
-    <t>geometry</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -217,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -252,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -428,53 +350,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>9</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DISTRICT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CD_uninsurance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CD_uninsurance_moe</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CD_pop</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>percentage_uninsured</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>percentage_uninsured_moe</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>within_sd</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>between_sd</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="B2">
         <v>12040</v>
@@ -498,235 +429,253 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>11</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="B3">
+        <v>10961</v>
+      </c>
+      <c r="C3">
+        <v>297</v>
+      </c>
+      <c r="D3">
+        <v>165808</v>
+      </c>
+      <c r="E3">
+        <v>6.6</v>
+      </c>
+      <c r="F3">
+        <v>0.2</v>
+      </c>
+      <c r="G3">
+        <v>4.4</v>
+      </c>
+      <c r="H3">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4">
         <v>8861</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>216</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <v>156728</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>5.7</v>
       </c>
-      <c r="F3">
+      <c r="F4">
         <v>0.1</v>
       </c>
-      <c r="G3">
+      <c r="G4">
         <v>3.7</v>
       </c>
-      <c r="H3">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4">
+      <c r="H4">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5">
         <v>10272</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>245</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>152603</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>6.7</v>
       </c>
-      <c r="F4">
-        <v>0.2</v>
-      </c>
-      <c r="G4">
+      <c r="F5">
+        <v>0.2</v>
+      </c>
+      <c r="G5">
         <v>4.3</v>
       </c>
-      <c r="H4">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
+      <c r="H5">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6">
         <v>7451</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>242</v>
       </c>
-      <c r="D5">
+      <c r="D6">
         <v>152871</v>
       </c>
-      <c r="E5">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="F5">
-        <v>0.2</v>
-      </c>
-      <c r="G5">
+      <c r="E6">
+        <v>4.9</v>
+      </c>
+      <c r="F6">
+        <v>0.2</v>
+      </c>
+      <c r="G6">
         <v>2.7</v>
       </c>
-      <c r="H5">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6">
+      <c r="H6">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7">
         <v>8945</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>255</v>
       </c>
-      <c r="D6">
+      <c r="D7">
         <v>163530</v>
       </c>
-      <c r="E6">
+      <c r="E7">
         <v>5.5</v>
       </c>
-      <c r="F6">
-        <v>0.2</v>
-      </c>
-      <c r="G6">
+      <c r="F7">
+        <v>0.2</v>
+      </c>
+      <c r="G7">
         <v>3.7</v>
       </c>
-      <c r="H6">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7">
+      <c r="H7">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8">
         <v>12244</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>261</v>
       </c>
-      <c r="D7">
+      <c r="D8">
         <v>166431</v>
       </c>
-      <c r="E7">
+      <c r="E8">
         <v>7.4</v>
       </c>
-      <c r="F7">
-        <v>0.2</v>
-      </c>
-      <c r="G7">
+      <c r="F8">
+        <v>0.2</v>
+      </c>
+      <c r="G8">
         <v>5.8</v>
       </c>
-      <c r="H7">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8">
+      <c r="H8">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9">
         <v>19202</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>321</v>
       </c>
-      <c r="D8">
+      <c r="D9">
         <v>163993</v>
       </c>
-      <c r="E8">
+      <c r="E9">
         <v>11.7</v>
       </c>
-      <c r="F8">
-        <v>0.2</v>
-      </c>
-      <c r="G8">
+      <c r="F9">
+        <v>0.2</v>
+      </c>
+      <c r="G9">
         <v>5.7</v>
       </c>
-      <c r="H8">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9">
+      <c r="H9">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10">
         <v>9672</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>230</v>
       </c>
-      <c r="D9">
+      <c r="D10">
         <v>155444</v>
       </c>
-      <c r="E9">
+      <c r="E10">
         <v>6.2</v>
       </c>
-      <c r="F9">
+      <c r="F10">
         <v>0.1</v>
       </c>
-      <c r="G9">
+      <c r="G10">
         <v>3.9</v>
       </c>
-      <c r="H9">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10">
+      <c r="H10">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B11">
         <v>16481</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>300</v>
       </c>
-      <c r="D10">
+      <c r="D11">
         <v>163206</v>
       </c>
-      <c r="E10">
+      <c r="E11">
         <v>10.1</v>
       </c>
-      <c r="F10">
-        <v>0.2</v>
-      </c>
-      <c r="G10">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="H10">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>10961</v>
-      </c>
-      <c r="C11">
-        <v>297</v>
-      </c>
-      <c r="D11">
-        <v>165808</v>
-      </c>
-      <c r="E11">
-        <v>6.6</v>
-      </c>
       <c r="F11">
         <v>0.2</v>
       </c>
       <c r="G11">
-        <v>4.4000000000000004</v>
+        <v>4.9</v>
       </c>
       <c r="H11">
         <v>2.1</v>

</xml_diff>